<commit_message>
Comp Intelligence: horizontal type chip-cloud (STI/MH) + rank estimate restored
- STI/MH long GMB-category list now renders as a horizontal wrapping chip cloud
  (full-width) instead of a tall vertical bar list; still multi-select + hide.
- Rank restored as an ESTIMATE from our SERP grid (serp_analyses allo_rank):
  new "Rank (est.)" column + 4-way verdict — Winning / Defend (rank #1 but
  out-reviewed) / Outrank (reviews but ranked below) / Build reviews.
  Falls back to review-only where grid rank is absent (most of MH).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Competition_Action_Plan.xlsx
+++ b/Competition_Action_Plan.xlsx
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Amravati</t>
+          <t>Indore</t>
         </is>
       </c>
       <c r="C60" s="4" t="n">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Shubham Hi-Tech Hospital and Test Tube Baby Centre 413 vs our median 3).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr Batra’s Homeopathy, Hair &amp; Skin Clinic 1517 vs our median 1).</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
@@ -3131,11 +3131,11 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>Shubham Hi-Tech Hospital and Test Tube Baby Centre (413)</t>
+          <t>Dr Batra’s Homeopathy, Hair &amp; Skin Clinic (1517)</t>
         </is>
       </c>
       <c r="I60" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" ht="40" customHeight="1">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Indore</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="C61" s="4" t="n">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Kurnool</t>
         </is>
       </c>
       <c r="C62" s="4" t="n">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr Batra’s Homeopathy, Hair &amp; Skin Clinic 1517 vs our median 1).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Vijaya Diagnostic Centre Kurnool (Gayathri Estate) - Pathology &amp; Radiology Lab | Full Body Checkup 18578 vs our median 12).</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -3217,11 +3217,11 @@
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>Dr Batra’s Homeopathy, Hair &amp; Skin Clinic (1517)</t>
+          <t>Vijaya Diagnostic Centre Kurnool (Gayathri Estate) - Pathology &amp; Radiology Lab | Full Body Checkup (18578)</t>
         </is>
       </c>
       <c r="I62" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="63" ht="40" customHeight="1">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Kurnool</t>
+          <t>MUMBAI</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Vijaya Diagnostic Centre Kurnool (Gayathri Estate) - Pathology &amp; Radiology Lab | Full Body Checkup 18578 vs our median 12).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Unique Diagnostic Centre 1202 vs our median 380).</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Vijaya Diagnostic Centre Kurnool (Gayathri Estate) - Pathology &amp; Radiology Lab | Full Body Checkup (18578)</t>
+          <t>Unique Diagnostic Centre (1202)</t>
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>12</v>
+        <v>380</v>
       </c>
     </row>
     <row r="64" ht="40" customHeight="1">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>MUMBAI</t>
+          <t>Rajkot</t>
         </is>
       </c>
       <c r="C64" s="4" t="n">
@@ -3293,7 +3293,7 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Unique Diagnostic Centre 1202 vs our median 380).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Bhatt Pathology Laboratory - Main Branch 5653 vs our median 0).</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -3303,11 +3303,11 @@
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>Unique Diagnostic Centre (1202)</t>
+          <t>Dr. Bhatt Pathology Laboratory - Main Branch (5653)</t>
         </is>
       </c>
       <c r="I64" s="4" t="n">
-        <v>380</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" ht="40" customHeight="1">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Raipur</t>
+          <t>Tumkur</t>
         </is>
       </c>
       <c r="C65" s="4" t="n">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Pathkind Labs 640 vs our median 2).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Indira IVF Fertility Centre in Tumkur - Best IVF Centre 156 vs our median 0).</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -3346,22 +3346,22 @@
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>Pathkind Labs (640)</t>
+          <t>Indira IVF Fertility Centre in Tumkur - Best IVF Centre (156)</t>
         </is>
       </c>
       <c r="I65" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" ht="40" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>Mental Health</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Rajkot</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="C66" s="4" t="n">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Bhatt Pathology Laboratory - Main Branch 5653 vs our median 0).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival GIPS Hospital and De-addiction Centre 15776 vs our median 29).</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
@@ -3389,22 +3389,22 @@
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>Dr. Bhatt Pathology Laboratory - Main Branch (5653)</t>
+          <t>GIPS Hospital and De-addiction Centre (15776)</t>
         </is>
       </c>
       <c r="I66" s="4" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="67" ht="40" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>Mental Health</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Ranchi</t>
+          <t>Amravati</t>
         </is>
       </c>
       <c r="C67" s="4" t="n">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Health Home 761 vs our median 392).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Vertex Healing Centre 483 vs our median 3).</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
@@ -3432,22 +3432,22 @@
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>Health Home (761)</t>
+          <t>Vertex Healing Centre (483)</t>
         </is>
       </c>
       <c r="I67" s="4" t="n">
-        <v>392</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68" ht="40" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>Mental Health</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Tumkur</t>
+          <t>Aurangabad</t>
         </is>
       </c>
       <c r="C68" s="4" t="n">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Indira IVF Fertility Centre in Tumkur - Best IVF Centre 156 vs our median 0).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Pranit Psychological Counseling &amp; Testing Center - IQ testing Aptitude &amp; career counseling in Aurangabad 1237 vs our median 53).</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -3475,22 +3475,22 @@
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>Indira IVF Fertility Centre in Tumkur - Best IVF Centre (156)</t>
+          <t>Pranit Psychological Counseling &amp; Testing Center - IQ testing Aptitude &amp; career counseling in Aurangabad (1237)</t>
         </is>
       </c>
       <c r="I68" s="4" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
     </row>
     <row r="69" ht="40" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>STI</t>
+          <t>Mental Health</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Vadodara</t>
+          <t>Bhopal</t>
         </is>
       </c>
       <c r="C69" s="4" t="n">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr Batra’s Homeopathy, Hair &amp; Skin Clinic 1497 vs our median 15).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Prayas Nasha Mukti evam Manochikitsa Kendra (Psychiatric Hospital &amp; Rehabilitation center)आयुष्मान योजना से निःशुल्क उपचार 1451 vs our median 16).</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr">
@@ -3518,11 +3518,11 @@
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>Dr Batra’s Homeopathy, Hair &amp; Skin Clinic (1497)</t>
+          <t>Prayas Nasha Mukti evam Manochikitsa Kendra (Psychiatric Hospital &amp; Rehabilitation center)आयुष्मान योजना से निःशुल्क उपचार (1451)</t>
         </is>
       </c>
       <c r="I69" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="70" ht="40" customHeight="1">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Gandhinagar</t>
         </is>
       </c>
       <c r="C70" s="4" t="n">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival GIPS Hospital and De-addiction Centre 15776 vs our median 29).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival SMVS Swaminarayan Hospital 15626 vs our median 15).</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
@@ -3561,11 +3561,11 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>GIPS Hospital and De-addiction Centre (15776)</t>
+          <t>SMVS Swaminarayan Hospital (15626)</t>
         </is>
       </c>
       <c r="I70" s="4" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71" ht="40" customHeight="1">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Amravati</t>
+          <t>Indore</t>
         </is>
       </c>
       <c r="C71" s="4" t="n">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Vertex Healing Centre 483 vs our median 3).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling 529 vs our median 1).</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr">
@@ -3604,11 +3604,11 @@
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>Vertex Healing Centre (483)</t>
+          <t>Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling (529)</t>
         </is>
       </c>
       <c r="I71" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" ht="40" customHeight="1">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Aurangabad</t>
+          <t>Kochi</t>
         </is>
       </c>
       <c r="C72" s="4" t="n">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Pranit Psychological Counseling &amp; Testing Center - IQ testing Aptitude &amp; career counseling in Aurangabad 1237 vs our median 53).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling 529 vs our median 1).</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
@@ -3647,11 +3647,11 @@
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>Pranit Psychological Counseling &amp; Testing Center - IQ testing Aptitude &amp; career counseling in Aurangabad (1237)</t>
+          <t>Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling (529)</t>
         </is>
       </c>
       <c r="I72" s="4" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" ht="40" customHeight="1">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Bhopal</t>
+          <t>Kurnool</t>
         </is>
       </c>
       <c r="C73" s="4" t="n">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Prayas Nasha Mukti evam Manochikitsa Kendra (Psychiatric Hospital &amp; Rehabilitation center)आयुष्मान योजना से निःशुल्क उपचार 1451 vs our median 16).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival YASH Relationship Centre (Lenin Perumalla Psychologist) 572 vs our median 12).</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -3690,11 +3690,11 @@
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Prayas Nasha Mukti evam Manochikitsa Kendra (Psychiatric Hospital &amp; Rehabilitation center)आयुष्मान योजना से निःशुल्क उपचार (1451)</t>
+          <t>YASH Relationship Centre (Lenin Perumalla Psychologist) (572)</t>
         </is>
       </c>
       <c r="I73" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="74" ht="40" customHeight="1">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Gandhinagar</t>
+          <t>MUMBAI</t>
         </is>
       </c>
       <c r="C74" s="4" t="n">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival SMVS Swaminarayan Hospital 15626 vs our median 15).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Vikas Deshmukh - Psychiatrist &amp; Sexologist in Navi Mumbai 624 vs our median 380).</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>SMVS Swaminarayan Hospital (15626)</t>
+          <t>Dr. Vikas Deshmukh - Psychiatrist &amp; Sexologist in Navi Mumbai (624)</t>
         </is>
       </c>
       <c r="I74" s="4" t="n">
-        <v>15</v>
+        <v>380</v>
       </c>
     </row>
     <row r="75" ht="40" customHeight="1">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Indore</t>
+          <t>Mangaluru</t>
         </is>
       </c>
       <c r="C75" s="4" t="n">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling 529 vs our median 1).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Birla Fertility &amp; IVF - Best IVF Centre in Mangalore, Karnataka 1244 vs our median 168).</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -3776,11 +3776,11 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling (529)</t>
+          <t>Birla Fertility &amp; IVF - Best IVF Centre in Mangalore, Karnataka (1244)</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
-        <v>1</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" ht="40" customHeight="1">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Nagpur</t>
         </is>
       </c>
       <c r="C76" s="4" t="n">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling 529 vs our median 1).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Sourabh Pal 592 vs our median 179).</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
@@ -3819,11 +3819,11 @@
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Fly Future Education | Best Overseas Education Consultant in Indore | MBBS in Abroad &amp; India | NEET Counselling (529)</t>
+          <t>Dr. Sourabh Pal (592)</t>
         </is>
       </c>
       <c r="I76" s="4" t="n">
-        <v>1</v>
+        <v>179</v>
       </c>
     </row>
     <row r="77" ht="40" customHeight="1">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Kurnool</t>
+          <t>Nashik</t>
         </is>
       </c>
       <c r="C77" s="4" t="n">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival YASH Relationship Centre (Lenin Perumalla Psychologist) 572 vs our median 12).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Sai Santosh Spine Cure centre--Ayush Height clinic=Dr Mitke| Best Ayurvedic Doctor in Nashik | spine specialist In Nashik 1382 vs our median 99).</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
@@ -3862,11 +3862,11 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>YASH Relationship Centre (Lenin Perumalla Psychologist) (572)</t>
+          <t>Sai Santosh Spine Cure centre--Ayush Height clinic=Dr Mitke| Best Ayurvedic Doctor in Nashik | spine specialist In Nashik (1382)</t>
         </is>
       </c>
       <c r="I77" s="4" t="n">
-        <v>12</v>
+        <v>99</v>
       </c>
     </row>
     <row r="78" ht="40" customHeight="1">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>MUMBAI</t>
+          <t>Raipur</t>
         </is>
       </c>
       <c r="C78" s="4" t="n">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Vikas Deshmukh - Psychiatrist &amp; Sexologist in Navi Mumbai 624 vs our median 380).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Bakhru's 2214 vs our median 2).</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Dr. Vikas Deshmukh - Psychiatrist &amp; Sexologist in Navi Mumbai (624)</t>
+          <t>Dr. Bakhru's (2214)</t>
         </is>
       </c>
       <c r="I78" s="4" t="n">
-        <v>380</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79" ht="40" customHeight="1">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Mangaluru</t>
+          <t>Rajkot</t>
         </is>
       </c>
       <c r="C79" s="4" t="n">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Birla Fertility &amp; IVF - Best IVF Centre in Mangalore, Karnataka 1244 vs our median 168).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Mind Care Hospital - Dr. Rajesh Ram Psychiatrist in Rajkot | De-Addiction specialist | Sexologist in Rajkot 1479 vs our median 0).</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
@@ -3948,11 +3948,11 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Birla Fertility &amp; IVF - Best IVF Centre in Mangalore, Karnataka (1244)</t>
+          <t>Mind Care Hospital - Dr. Rajesh Ram Psychiatrist in Rajkot | De-Addiction specialist | Sexologist in Rajkot (1479)</t>
         </is>
       </c>
       <c r="I79" s="4" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" ht="40" customHeight="1">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Ranchi</t>
         </is>
       </c>
       <c r="C80" s="4" t="n">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Sourabh Pal 592 vs our median 179).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Paramarsh Bharti 994 vs our median 392).</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr">
@@ -3991,11 +3991,11 @@
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>Dr. Sourabh Pal (592)</t>
+          <t>Paramarsh Bharti (994)</t>
         </is>
       </c>
       <c r="I80" s="4" t="n">
-        <v>179</v>
+        <v>392</v>
       </c>
     </row>
     <row r="81" ht="40" customHeight="1">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Nashik</t>
+          <t>Surat</t>
         </is>
       </c>
       <c r="C81" s="4" t="n">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Sai Santosh Spine Cure centre--Ayush Height clinic=Dr Mitke| Best Ayurvedic Doctor in Nashik | spine specialist In Nashik 1382 vs our median 99).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Best Career Counselling 948 vs our median 33).</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
@@ -4034,11 +4034,11 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>Sai Santosh Spine Cure centre--Ayush Height clinic=Dr Mitke| Best Ayurvedic Doctor in Nashik | spine specialist In Nashik (1382)</t>
+          <t>Best Career Counselling (948)</t>
         </is>
       </c>
       <c r="I81" s="4" t="n">
-        <v>99</v>
+        <v>33</v>
       </c>
     </row>
     <row r="82" ht="40" customHeight="1">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Raipur</t>
+          <t>Tumkur</t>
         </is>
       </c>
       <c r="C82" s="4" t="n">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Dr. Bakhru's 2214 vs our median 2).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Siddaganga Medical College &amp; Research Institute 1139 vs our median 0).</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
@@ -4077,11 +4077,11 @@
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>Dr. Bakhru's (2214)</t>
+          <t>Siddaganga Medical College &amp; Research Institute (1139)</t>
         </is>
       </c>
       <c r="I82" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" ht="40" customHeight="1">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Rajkot</t>
+          <t>Vadodara</t>
         </is>
       </c>
       <c r="C83" s="4" t="n">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Mind Care Hospital - Dr. Rajesh Ram Psychiatrist in Rajkot | De-Addiction specialist | Sexologist in Rajkot 1479 vs our median 0).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Psychiatrist Dr Kritagnasinh vaghela JAY CLINIC 1150 vs our median 15).</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
@@ -4120,11 +4120,11 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Mind Care Hospital - Dr. Rajesh Ram Psychiatrist in Rajkot | De-Addiction specialist | Sexologist in Rajkot (1479)</t>
+          <t>Psychiatrist Dr Kritagnasinh vaghela JAY CLINIC (1150)</t>
         </is>
       </c>
       <c r="I83" s="4" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="84" ht="40" customHeight="1">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Ranchi</t>
+          <t>Visakhapatnam</t>
         </is>
       </c>
       <c r="C84" s="4" t="n">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Paramarsh Bharti 994 vs our median 392).</t>
+          <t>No paid spend. 1/1 clinics out-reviewed (top rival Travancore Ayurveda NABH Panchakarma Clinic | MVP Colony | Vizag 720 vs our median 41).</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
@@ -4163,182 +4163,10 @@
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>Paramarsh Bharti (994)</t>
+          <t>Travancore Ayurveda NABH Panchakarma Clinic | MVP Colony | Vizag (720)</t>
         </is>
       </c>
       <c r="I84" s="4" t="n">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>Mental Health</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>Surat</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D85" s="12" t="inlineStr">
-        <is>
-          <t>ORGANIC</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>Reviews / GMB</t>
-        </is>
-      </c>
-      <c r="F85" s="6" t="inlineStr">
-        <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Best Career Counselling 948 vs our median 33).</t>
-        </is>
-      </c>
-      <c r="G85" s="6" t="inlineStr">
-        <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
-        </is>
-      </c>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>Best Career Counselling (948)</t>
-        </is>
-      </c>
-      <c r="I85" s="4" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="86" ht="40" customHeight="1">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>Mental Health</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>Tumkur</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D86" s="12" t="inlineStr">
-        <is>
-          <t>ORGANIC</t>
-        </is>
-      </c>
-      <c r="E86" s="4" t="inlineStr">
-        <is>
-          <t>Reviews / GMB</t>
-        </is>
-      </c>
-      <c r="F86" s="6" t="inlineStr">
-        <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Siddaganga Medical College &amp; Research Institute 1139 vs our median 0).</t>
-        </is>
-      </c>
-      <c r="G86" s="6" t="inlineStr">
-        <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
-        </is>
-      </c>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>Siddaganga Medical College &amp; Research Institute (1139)</t>
-        </is>
-      </c>
-      <c r="I86" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" ht="40" customHeight="1">
-      <c r="A87" s="3" t="inlineStr">
-        <is>
-          <t>Mental Health</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="inlineStr">
-        <is>
-          <t>Vadodara</t>
-        </is>
-      </c>
-      <c r="C87" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D87" s="12" t="inlineStr">
-        <is>
-          <t>ORGANIC</t>
-        </is>
-      </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>Reviews / GMB</t>
-        </is>
-      </c>
-      <c r="F87" s="6" t="inlineStr">
-        <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Psychiatrist Dr Kritagnasinh vaghela JAY CLINIC 1150 vs our median 15).</t>
-        </is>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
-        </is>
-      </c>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>Psychiatrist Dr Kritagnasinh vaghela JAY CLINIC (1150)</t>
-        </is>
-      </c>
-      <c r="I87" s="4" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="88" ht="40" customHeight="1">
-      <c r="A88" s="3" t="inlineStr">
-        <is>
-          <t>Mental Health</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>Visakhapatnam</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D88" s="12" t="inlineStr">
-        <is>
-          <t>ORGANIC</t>
-        </is>
-      </c>
-      <c r="E88" s="4" t="inlineStr">
-        <is>
-          <t>Reviews / GMB</t>
-        </is>
-      </c>
-      <c r="F88" s="6" t="inlineStr">
-        <is>
-          <t>No paid spend. 1/1 clinics out-reviewed (top rival Travancore Ayurveda NABH Panchakarma Clinic | MVP Colony | Vizag 720 vs our median 41).</t>
-        </is>
-      </c>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
-        </is>
-      </c>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>Travancore Ayurveda NABH Panchakarma Clinic | MVP Colony | Vizag (720)</t>
-        </is>
-      </c>
-      <c r="I88" s="4" t="n">
         <v>41</v>
       </c>
     </row>
@@ -6982,7 +6810,7 @@
         <v>19.9</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="S3" s="6" t="inlineStr">
         <is>
@@ -7053,7 +6881,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
@@ -7124,7 +6952,7 @@
         <v>7</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
@@ -7266,7 +7094,7 @@
         <v>7</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="inlineStr">
         <is>
@@ -7408,7 +7236,7 @@
         <v>6</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" s="6" t="inlineStr">
         <is>
@@ -7479,7 +7307,7 @@
         <v>544</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" s="6" t="inlineStr">
         <is>
@@ -7621,7 +7449,7 @@
         <v>67.40000000000001</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" s="6" t="inlineStr">
         <is>
@@ -7692,7 +7520,7 @@
         <v>13.1</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" s="6" t="inlineStr">
         <is>
@@ -7834,7 +7662,7 @@
         <v>127.9</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" s="6" t="inlineStr">
         <is>
@@ -7905,7 +7733,7 @@
         <v>21.4</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" s="6" t="inlineStr">
         <is>
@@ -8118,7 +7946,7 @@
         <v>1.5</v>
       </c>
       <c r="R19" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" s="6" t="inlineStr">
         <is>
@@ -8331,7 +8159,7 @@
         <v>330.7</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" s="6" t="inlineStr">
         <is>
@@ -8544,7 +8372,7 @@
         <v>4.9</v>
       </c>
       <c r="R25" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" s="6" t="inlineStr">
         <is>
@@ -9167,7 +8995,7 @@
         <v>40</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="S3" s="6" t="inlineStr">
         <is>
@@ -9238,7 +9066,7 @@
         <v>64.2</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
@@ -9309,7 +9137,7 @@
         <v>28</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
@@ -9380,7 +9208,7 @@
         <v>12.2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" s="6" t="inlineStr">
         <is>
@@ -9451,7 +9279,7 @@
         <v>4.6</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S7" s="6" t="inlineStr">
         <is>
@@ -9522,7 +9350,7 @@
         <v>39.9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="S8" s="6" t="inlineStr">
         <is>
@@ -9593,7 +9421,7 @@
         <v>37.6</v>
       </c>
       <c r="R9" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="inlineStr">
         <is>
@@ -9664,7 +9492,7 @@
         <v>1.4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" s="6" t="inlineStr">
         <is>
@@ -9735,7 +9563,7 @@
         <v>544</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" s="6" t="inlineStr">
         <is>
@@ -9806,7 +9634,7 @@
         <v>37.8</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" s="6" t="inlineStr">
         <is>
@@ -9877,7 +9705,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" s="6" t="inlineStr">
         <is>
@@ -9948,7 +9776,7 @@
         <v>49.9</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" s="6" t="inlineStr">
         <is>
@@ -10019,7 +9847,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" s="6" t="inlineStr">
         <is>
@@ -10090,7 +9918,7 @@
         <v>35.2</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" s="6" t="inlineStr">
         <is>
@@ -10161,7 +9989,7 @@
         <v>4.7</v>
       </c>
       <c r="R17" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17" s="6" t="inlineStr">
         <is>
@@ -10232,7 +10060,7 @@
         <v>67.40000000000001</v>
       </c>
       <c r="R18" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S18" s="6" t="inlineStr">
         <is>
@@ -10303,7 +10131,7 @@
         <v>13.8</v>
       </c>
       <c r="R19" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" s="6" t="inlineStr">
         <is>
@@ -10445,7 +10273,7 @@
         <v>20.5</v>
       </c>
       <c r="R21" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21" s="6" t="inlineStr">
         <is>
@@ -10516,11 +10344,11 @@
         <v>137.7</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" s="6" t="inlineStr">
         <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
+          <t>Holding on reviews organically.</t>
         </is>
       </c>
     </row>
@@ -10855,11 +10683,11 @@
         <v>320</v>
       </c>
       <c r="R27" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" s="6" t="inlineStr">
         <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
+          <t>Holding on reviews organically.</t>
         </is>
       </c>
     </row>
@@ -10997,11 +10825,11 @@
         <v>1.9</v>
       </c>
       <c r="R29" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" s="6" t="inlineStr">
         <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
+          <t>Holding on reviews organically.</t>
         </is>
       </c>
     </row>
@@ -11139,11 +10967,11 @@
         <v>99.8</v>
       </c>
       <c r="R31" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" s="6" t="inlineStr">
         <is>
-          <t>Organic/GMB market — build reviews &amp; GMB before/instead of paid.</t>
+          <t>Holding on reviews organically.</t>
         </is>
       </c>
     </row>
@@ -11352,7 +11180,7 @@
         <v>23.1</v>
       </c>
       <c r="R3" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="S3" s="6" t="inlineStr">
         <is>
@@ -11423,7 +11251,7 @@
         <v>11.3</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
@@ -11494,7 +11322,7 @@
         <v>36.9</v>
       </c>
       <c r="R5" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
@@ -11707,7 +11535,7 @@
         <v>29.9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" s="6" t="inlineStr">
         <is>
@@ -13473,7 +13301,7 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (1062 vs 29)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1062 vs 29)</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -13523,7 +13351,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (435 vs 3)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (435 vs 3)</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -13573,7 +13401,7 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (259 vs 53)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (259 vs 53)</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -13621,12 +13449,12 @@
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -13721,12 +13549,12 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -13769,12 +13597,12 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -13869,7 +13697,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (931 vs 9)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (931 vs 9)</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -13919,7 +13747,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Unani rival leads 536 vs 492</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (536 vs 492)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -14069,7 +13897,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (616 vs 9)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (616 vs 9)</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -14217,7 +14045,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Ayurvedic rival far ahead (1396 vs 47)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1396 vs 47)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -14267,7 +14095,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (828 vs 47)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (828 vs 47)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -14317,7 +14145,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Ayurvedic rival far ahead (1396 vs 478)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1396 vs 478)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -14465,7 +14293,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Homeopathic rival far ahead (1078 vs 16)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1078 vs 16)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -14563,7 +14391,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (2242 vs 594)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2242 vs 594)</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -14713,7 +14541,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (924 vs 320)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (924 vs 320)</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -14813,7 +14641,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (149 vs 44)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (149 vs 44)</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -14963,7 +14791,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (57 vs 15)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (57 vs 15)</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -15063,7 +14891,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Unani rival far ahead (2119 vs 947)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2119 vs 947)</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -15113,7 +14941,7 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Unani rival far ahead (2119 vs 947)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2119 vs 947)</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr">
@@ -15209,7 +15037,7 @@
       <c r="J38" s="4" t="inlineStr"/>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival leads 354 vs 329</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (354 vs 329)</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr">
@@ -15259,7 +15087,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (467 vs 9)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (467 vs 9)</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -15309,7 +15137,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Homeopathic rival far ahead (1016 vs 9)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1016 vs 9)</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -15359,12 +15187,12 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -15409,7 +15237,7 @@
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (2375 vs 187)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2375 vs 187)</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
@@ -15459,7 +15287,7 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival leads 354 vs 329</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (354 vs 329)</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr">
@@ -15705,7 +15533,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (536 vs 90)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (536 vs 90)</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr">
@@ -15899,7 +15727,7 @@
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Unani rival leads 256 vs 168</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (256 vs 168)</t>
         </is>
       </c>
       <c r="L52" s="6" t="inlineStr">
@@ -16047,12 +15875,12 @@
       <c r="J55" s="4" t="inlineStr"/>
       <c r="K55" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L55" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -16297,12 +16125,12 @@
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>Winning — hold + keep reviews</t>
+          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr">
         <is>
-          <t>Hold + keep reviews</t>
+          <t>Fix GMB rank/bid (we have reviews)</t>
         </is>
       </c>
     </row>
@@ -16847,7 +16675,7 @@
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (248 vs 81)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (248 vs 81)</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr">
@@ -16897,12 +16725,12 @@
       </c>
       <c r="K72" s="6" t="inlineStr">
         <is>
-          <t>Winning — hold + keep reviews</t>
+          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
         </is>
       </c>
       <c r="L72" s="6" t="inlineStr">
         <is>
-          <t>Hold + keep reviews</t>
+          <t>Fix GMB rank/bid (we have reviews)</t>
         </is>
       </c>
     </row>
@@ -16947,7 +16775,7 @@
       </c>
       <c r="K73" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (2139 vs 449)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2139 vs 449)</t>
         </is>
       </c>
       <c r="L73" s="6" t="inlineStr">
@@ -17097,7 +16925,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Homeopathic rival far ahead (1775 vs 356)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1775 vs 356)</t>
         </is>
       </c>
       <c r="L76" s="6" t="inlineStr">
@@ -17147,7 +16975,7 @@
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (865 vs 305)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (865 vs 305)</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr">
@@ -17295,12 +17123,12 @@
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>Winning — hold + keep reviews</t>
+          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
         </is>
       </c>
       <c r="L80" s="6" t="inlineStr">
         <is>
-          <t>Hold + keep reviews</t>
+          <t>Fix GMB rank/bid (we have reviews)</t>
         </is>
       </c>
     </row>
@@ -17345,7 +17173,7 @@
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Ayurvedic rival far ahead (706 vs 33)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (706 vs 33)</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr">
@@ -17443,7 +17271,7 @@
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Allopathic rival far ahead (1919 vs 15)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1919 vs 15)</t>
         </is>
       </c>
       <c r="L83" s="6" t="inlineStr">
@@ -17643,7 +17471,7 @@
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Psychiatrist rival far ahead (15775 vs 29)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (15775 vs 29)</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -17693,7 +17521,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Fertility clinic rival far ahead (413 vs 3)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (413 vs 3)</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -17841,7 +17669,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Fertility clinic rival far ahead (884 vs 9)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (884 vs 9)</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -17891,7 +17719,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (1932 vs 338)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1932 vs 338)</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -17991,7 +17819,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (6449 vs 655)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (6449 vs 655)</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -18041,7 +17869,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (18997 vs 492)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (18997 vs 492)</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -18091,7 +17919,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (18997 vs 45)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (18997 vs 45)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -18141,7 +17969,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (18997 vs 338)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (18997 vs 338)</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -18191,7 +18019,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival far ahead (5744 vs 385)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (5744 vs 385)</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -18241,7 +18069,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (842 vs 198)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (842 vs 198)</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -18291,7 +18119,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (18997 vs 338)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (18997 vs 338)</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -18389,7 +18217,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (21686 vs 627)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (21686 vs 627)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -18439,7 +18267,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (21686 vs 47)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (21686 vs 47)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -18489,7 +18317,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (21686 vs 47)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (21686 vs 47)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -18539,7 +18367,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Sexologist rival far ahead (1396 vs 478)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1396 vs 478)</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -18589,7 +18417,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival leads 861 vs 604</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (861 vs 604)</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -18687,7 +18515,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Sexologist rival far ahead (1078 vs 16)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1078 vs 16)</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -18785,7 +18613,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical laboratory rival far ahead (1238 vs 594)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1238 vs 594)</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -18835,7 +18663,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical laboratory rival far ahead (1238 vs 320)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1238 vs 320)</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -18885,7 +18713,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (851 vs 3)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (851 vs 3)</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr">
@@ -18935,7 +18763,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (4337 vs 320)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (4337 vs 320)</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr">
@@ -18985,7 +18813,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (8968 vs 148)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (8968 vs 148)</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr">
@@ -19035,7 +18863,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (1190 vs 44)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1190 vs 44)</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -19085,7 +18913,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival far ahead (6775 vs 594)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (6775 vs 594)</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr">
@@ -19135,7 +18963,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Blood testing service rival leads 413 vs 288</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (413 vs 288)</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -19185,7 +19013,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — General hospital rival far ahead (567 vs 15)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (567 vs 15)</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr">
@@ -19235,7 +19063,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Doctor rival far ahead (635 vs 31)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (635 vs 31)</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -19285,7 +19113,7 @@
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (10590 vs 947)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (10590 vs 947)</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr">
@@ -19335,7 +19163,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (4637 vs 947)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (4637 vs 947)</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr">
@@ -19383,7 +19211,7 @@
       <c r="J38" s="4" t="inlineStr"/>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Sexologist rival far ahead (1459 vs 10)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1459 vs 10)</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr">
@@ -19431,7 +19259,7 @@
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (6238 vs 329)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (6238 vs 329)</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr">
@@ -19481,7 +19309,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (1894 vs 438)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1894 vs 438)</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr">
@@ -19531,7 +19359,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (3827 vs 9)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (3827 vs 9)</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr">
@@ -19581,7 +19409,7 @@
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival far ahead (4992 vs 990)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (4992 vs 990)</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
@@ -19631,7 +19459,7 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (2134 vs 187)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2134 vs 187)</t>
         </is>
       </c>
       <c r="L43" s="6" t="inlineStr">
@@ -19779,7 +19607,7 @@
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (7413 vs 73)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (7413 vs 73)</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr">
@@ -19829,7 +19657,7 @@
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (9270 vs 73)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (9270 vs 73)</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr">
@@ -19927,7 +19755,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (1096 vs 90)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1096 vs 90)</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr">
@@ -20121,7 +19949,7 @@
       </c>
       <c r="K53" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (785 vs 168)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (785 vs 168)</t>
         </is>
       </c>
       <c r="L53" s="6" t="inlineStr">
@@ -20171,7 +19999,7 @@
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival leads 1066 vs 712</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1066 vs 712)</t>
         </is>
       </c>
       <c r="L54" s="6" t="inlineStr">
@@ -20221,7 +20049,7 @@
       </c>
       <c r="K55" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival far ahead (1228 vs 380)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1228 vs 380)</t>
         </is>
       </c>
       <c r="L55" s="6" t="inlineStr">
@@ -20319,7 +20147,7 @@
       </c>
       <c r="K57" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (15414 vs 382)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (15414 vs 382)</t>
         </is>
       </c>
       <c r="L57" s="6" t="inlineStr">
@@ -20369,7 +20197,7 @@
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival far ahead (6925 vs 495)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (6925 vs 495)</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr">
@@ -20469,7 +20297,7 @@
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (15414 vs 197)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (15414 vs 197)</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr">
@@ -20519,7 +20347,7 @@
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival leads 803 vs 550</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (803 vs 550)</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr">
@@ -20619,7 +20447,7 @@
       </c>
       <c r="K63" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Sexologist rival far ahead (488 vs 10)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (488 vs 10)</t>
         </is>
       </c>
       <c r="L63" s="6" t="inlineStr">
@@ -20669,7 +20497,7 @@
       </c>
       <c r="K64" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival leads 563 vs 515</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (563 vs 515)</t>
         </is>
       </c>
       <c r="L64" s="6" t="inlineStr">
@@ -20769,7 +20597,7 @@
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical clinic rival far ahead (4866 vs 550)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (4866 vs 550)</t>
         </is>
       </c>
       <c r="L66" s="6" t="inlineStr">
@@ -20819,7 +20647,7 @@
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Sexologist rival far ahead (1566 vs 179)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1566 vs 179)</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr">
@@ -20869,7 +20697,7 @@
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical clinic rival far ahead (4937 vs 99)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (4937 vs 99)</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr">
@@ -20919,7 +20747,7 @@
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical diagnostic imaging center rival far ahead (1045 vs 260)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1045 vs 260)</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr">
@@ -20969,7 +20797,7 @@
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (691 vs 66)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (691 vs 66)</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr">
@@ -21019,7 +20847,7 @@
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — STD testing service rival far ahead (1202 vs 380)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1202 vs 380)</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr">
@@ -21069,7 +20897,7 @@
       </c>
       <c r="K72" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Homeopath rival far ahead (704 vs 81)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (704 vs 81)</t>
         </is>
       </c>
       <c r="L72" s="6" t="inlineStr">
@@ -21169,7 +20997,7 @@
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (11472 vs 449)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (11472 vs 449)</t>
         </is>
       </c>
       <c r="L74" s="6" t="inlineStr">
@@ -21269,7 +21097,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (2991 vs 330)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (2991 vs 330)</t>
         </is>
       </c>
       <c r="L76" s="6" t="inlineStr">
@@ -21319,7 +21147,7 @@
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (3234 vs 356)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (3234 vs 356)</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr">
@@ -21369,7 +21197,7 @@
       </c>
       <c r="K78" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical laboratory rival far ahead (4987 vs 305)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (4987 vs 305)</t>
         </is>
       </c>
       <c r="L78" s="6" t="inlineStr">
@@ -21419,7 +21247,7 @@
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival far ahead (640 vs 2)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (640 vs 2)</t>
         </is>
       </c>
       <c r="L79" s="6" t="inlineStr">
@@ -21517,7 +21345,7 @@
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Diagnostic center rival leads 761 vs 392</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (761 vs 392)</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr">
@@ -21567,7 +21395,7 @@
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — HIV testing center rival far ahead (1162 vs 33)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1162 vs 33)</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr">
@@ -21665,7 +21493,7 @@
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Homeopath rival far ahead (1497 vs 15)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (1497 vs 15)</t>
         </is>
       </c>
       <c r="L84" s="6" t="inlineStr">
@@ -21715,7 +21543,7 @@
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Specialized clinic rival far ahead (567 vs 41)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (567 vs 41)</t>
         </is>
       </c>
       <c r="L85" s="6" t="inlineStr">
@@ -22313,7 +22141,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Medical clinic rival leads 757 vs 746</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (757 vs 746)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -22811,7 +22639,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Hospital rival leads 719 vs 604</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (719 vs 604)</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -23357,7 +23185,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Psychiatrist rival far ahead (3253 vs 288)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (3253 vs 288)</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr">
@@ -23457,7 +23285,7 @@
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Psychiatrist rival far ahead (928 vs 31)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (928 vs 31)</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
@@ -24591,12 +24419,12 @@
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -24991,12 +24819,12 @@
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>OUTRANK — we have the reviews, fix GMB/bid</t>
+          <t>Winning — hold + keep reviews</t>
         </is>
       </c>
       <c r="L66" s="6" t="inlineStr">
         <is>
-          <t>Fix GMB rank/bid (we have reviews)</t>
+          <t>Hold + keep reviews</t>
         </is>
       </c>
     </row>
@@ -25391,7 +25219,7 @@
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>BUILD REVIEWS — Hospital rival far ahead (11251 vs 449)</t>
+          <t>DEFEND — rank ~#1 but out-reviewed (11251 vs 449)</t>
         </is>
       </c>
       <c r="L74" s="6" t="inlineStr">

</xml_diff>